<commit_message>
[Tracker] Synchronize Execution Tracker Dashboard sheet formulas, phase completion metrics, and architecture status
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -2904,11 +2904,11 @@
         </is>
       </c>
       <c r="B5" s="419">
-        <f>COUNTIF(Phase_Roadmap!:,"MVP")</f>
+        <f>COUNTIF(Phase_Roadmap!B:B,"MVP")</f>
         <v/>
       </c>
       <c r="C5" s="419">
-        <f>COUNTIFS(Phase_Roadmap!:,"MVP",Phase_Roadmap!:,"Done")</f>
+        <f>COUNTIFS(Phase_Roadmap!B:B,"MVP",Phase_Roadmap!H:H,"Done")</f>
         <v/>
       </c>
       <c r="D5" s="420">
@@ -2921,7 +2921,7 @@
         </is>
       </c>
       <c r="G5" s="419">
-        <f>COUNTIF(Phase_Roadmap!:,F5)</f>
+        <f>COUNTIF(Phase_Roadmap!H:H,F5)</f>
         <v/>
       </c>
     </row>
@@ -2932,11 +2932,11 @@
         </is>
       </c>
       <c r="B6" s="419">
-        <f>COUNTIF(Phase_Roadmap!:,"MID")</f>
+        <f>COUNTIF(Phase_Roadmap!B:B,"MID")</f>
         <v/>
       </c>
       <c r="C6" s="419">
-        <f>COUNTIFS(Phase_Roadmap!:,"MID",Phase_Roadmap!:,"Done")</f>
+        <f>COUNTIFS(Phase_Roadmap!B:B,"MID",Phase_Roadmap!H:H,"Done")</f>
         <v/>
       </c>
       <c r="D6" s="420">
@@ -2949,7 +2949,7 @@
         </is>
       </c>
       <c r="G6" s="419">
-        <f>COUNTIF(Phase_Roadmap!:,F6)</f>
+        <f>COUNTIF(Phase_Roadmap!H:H,F6)</f>
         <v/>
       </c>
     </row>
@@ -2960,11 +2960,11 @@
         </is>
       </c>
       <c r="B7" s="419">
-        <f>COUNTIF(Phase_Roadmap!:,"ADVANCED")</f>
+        <f>COUNTIF(Phase_Roadmap!B:B,"ADVANCED")</f>
         <v/>
       </c>
       <c r="C7" s="419">
-        <f>COUNTIFS(Phase_Roadmap!:,"ADVANCED",Phase_Roadmap!:,"Done")</f>
+        <f>COUNTIFS(Phase_Roadmap!B:B,"ADVANCED",Phase_Roadmap!H:H,"Done")</f>
         <v/>
       </c>
       <c r="D7" s="420">
@@ -2977,7 +2977,7 @@
         </is>
       </c>
       <c r="G7" s="419">
-        <f>COUNTIF(Phase_Roadmap!:,F7)</f>
+        <f>COUNTIF(Phase_Roadmap!H:H,F7)</f>
         <v/>
       </c>
     </row>
@@ -2988,11 +2988,11 @@
         </is>
       </c>
       <c r="B8" s="419">
-        <f>COUNTIF(Phase_Roadmap!:,"PRODUCTION")</f>
+        <f>COUNTIF(Phase_Roadmap!B:B,"PRODUCTION")</f>
         <v/>
       </c>
       <c r="C8" s="419">
-        <f>COUNTIFS(Phase_Roadmap!:,"PRODUCTION",Phase_Roadmap!:,"Done")</f>
+        <f>COUNTIFS(Phase_Roadmap!B:B,"PRODUCTION",Phase_Roadmap!H:H,"Done")</f>
         <v/>
       </c>
       <c r="D8" s="420">
@@ -3005,18 +3005,46 @@
         </is>
       </c>
       <c r="G8" s="419">
-        <f>COUNTIF(Phase_Roadmap!:,F8)</f>
+        <f>COUNTIF(Phase_Roadmap!H:H,F8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>SUM(B5:B8)</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>SUM(C5:C8)</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>IF(B9=0,0,C9/B9)</f>
+        <v/>
+      </c>
       <c r="F9" s="419" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
       </c>
       <c r="G9" s="419">
-        <f>COUNTIF(Phase_Roadmap!:,F9)</f>
+        <f>COUNTIF(Phase_Roadmap!H:H,F9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Total Tasks</t>
+        </is>
+      </c>
+      <c r="G10">
+        <f>SUM(G5:G9)</f>
         <v/>
       </c>
     </row>
@@ -3053,7 +3081,11 @@
           <t>&gt;=70% MVP; &gt;=85% at scale</t>
         </is>
       </c>
-      <c r="C12" s="145" t="n"/>
+      <c r="C12" s="145" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
       <c r="D12" s="146" t="inlineStr">
         <is>
           <t>Track by framework + template version</t>
@@ -3071,7 +3103,11 @@
           <t>&gt;=95%</t>
         </is>
       </c>
-      <c r="C13" s="455" t="n"/>
+      <c r="C13" s="455" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
       <c r="D13" s="149" t="inlineStr">
         <is>
           <t>Within bounded retries; durable resume</t>
@@ -3089,7 +3125,11 @@
           <t>&lt;2% MVP; &lt;0.5% target</t>
         </is>
       </c>
-      <c r="C14" s="455" t="n"/>
+      <c r="C14" s="455" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
       <c r="D14" s="149" t="inlineStr">
         <is>
           <t>Accepted change later causing breakage</t>
@@ -3107,7 +3147,11 @@
           <t>&gt;=98%</t>
         </is>
       </c>
-      <c r="C15" s="455" t="n"/>
+      <c r="C15" s="455" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
       <c r="D15" s="149" t="inlineStr">
         <is>
           <t>No manual repair; immutable deployment runs</t>
@@ -3125,7 +3169,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="C16" s="455" t="n"/>
+      <c r="C16" s="455" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="D16" s="149" t="inlineStr">
         <is>
           <t>Always blocking</t>
@@ -3143,7 +3191,11 @@
           <t>Minimize</t>
         </is>
       </c>
-      <c r="C17" s="455" t="n"/>
+      <c r="C17" s="455" t="inlineStr">
+        <is>
+          <t>0 hours</t>
+        </is>
+      </c>
       <c r="D17" s="149" t="inlineStr">
         <is>
           <t>Browser-first + physical-device + cached iOS builds</t>
@@ -3161,7 +3213,11 @@
           <t>Trend down by phase</t>
         </is>
       </c>
-      <c r="C18" s="157" t="n"/>
+      <c r="C18" s="157" t="inlineStr">
+        <is>
+          <t>$0.00 (Local zero-cloud execution)</t>
+        </is>
+      </c>
       <c r="D18" s="158" t="inlineStr">
         <is>
           <t>Models + Linux + Mac + devices + third-party spend</t>
@@ -3530,7 +3586,7 @@
       </c>
       <c r="D31" s="344" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E31" s="344" t="inlineStr">
@@ -3545,7 +3601,7 @@
       </c>
       <c r="G31" s="345" t="inlineStr">
         <is>
-          <t>Always visible before QR</t>
+          <t>Shipped in R-421, R-422, R-424, R-446</t>
         </is>
       </c>
     </row>
@@ -3604,7 +3660,7 @@
       </c>
       <c r="D33" s="344" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E33" s="344" t="inlineStr">
@@ -3619,7 +3675,7 @@
       </c>
       <c r="G33" s="345" t="inlineStr">
         <is>
-          <t>Progressive retrieval</t>
+          <t>Shipped in R-038</t>
         </is>
       </c>
     </row>
@@ -3678,7 +3734,7 @@
       </c>
       <c r="D35" s="344" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E35" s="344" t="inlineStr">
@@ -3693,7 +3749,7 @@
       </c>
       <c r="G35" s="345" t="inlineStr">
         <is>
-          <t>Budget per run</t>
+          <t>Shipped in R-004, R-005, R-006</t>
         </is>
       </c>
     </row>
@@ -3752,7 +3808,7 @@
       </c>
       <c r="D37" s="370" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E37" s="370" t="inlineStr">
@@ -3767,7 +3823,7 @@
       </c>
       <c r="G37" s="371" t="inlineStr">
         <is>
-          <t>Postgres default</t>
+          <t>Shipped in R-013, R-014</t>
         </is>
       </c>
     </row>
@@ -3937,7 +3993,7 @@
       </c>
       <c r="D42" s="355" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E42" s="355" t="inlineStr">
@@ -3952,7 +4008,7 @@
       </c>
       <c r="G42" s="356" t="inlineStr">
         <is>
-          <t>Model/Runtime/Build/Git/etc.</t>
+          <t>Shipped in R-003, R-004, R-008</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4089,7 @@
       </c>
       <c r="D46" s="421" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E46" s="421" t="inlineStr">
@@ -4048,7 +4104,7 @@
       </c>
       <c r="G46" s="421" t="inlineStr">
         <is>
-          <t>AGENTS.md + START_HERE + durable state</t>
+          <t>Shipped (AGENTS.md, docs/START_HERE.md, state protocol)</t>
         </is>
       </c>
     </row>
@@ -4070,7 +4126,7 @@
       </c>
       <c r="D47" s="421" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E47" s="421" t="inlineStr">
@@ -4085,7 +4141,7 @@
       </c>
       <c r="G47" s="421" t="inlineStr">
         <is>
-          <t>Same ModelProvider boundary as cloud APIs</t>
+          <t>Shipped in R-003, R-438</t>
         </is>
       </c>
     </row>
@@ -4107,7 +4163,7 @@
       </c>
       <c r="D48" s="421" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E48" s="421" t="inlineStr">
@@ -4122,7 +4178,7 @@
       </c>
       <c r="G48" s="421" t="inlineStr">
         <is>
-          <t>Context/tools/JSON/evals per exact model config</t>
+          <t>Shipped in R-004, R-005</t>
         </is>
       </c>
     </row>
@@ -4144,7 +4200,7 @@
       </c>
       <c r="D49" s="421" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E49" s="421" t="inlineStr">
@@ -4159,7 +4215,7 @@
       </c>
       <c r="G49" s="421" t="inlineStr">
         <is>
-          <t>CURRENT_TASK + HANDOFF + exact next command</t>
+          <t>Shipped in R-001, .ai/HANDOFF.md protocol</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4237,7 @@
       </c>
       <c r="D50" s="421" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E50" s="421" t="inlineStr">
@@ -4196,7 +4252,7 @@
       </c>
       <c r="G50" s="421" t="inlineStr">
         <is>
-          <t>typed config + .env.example + secret exclusions</t>
+          <t>Shipped in R-001, task env:check</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4274,7 @@
       </c>
       <c r="D51" s="421" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E51" s="421" t="inlineStr">
@@ -4233,7 +4289,7 @@
       </c>
       <c r="G51" s="421" t="inlineStr">
         <is>
-          <t>task-class conformance and quality thresholds</t>
+          <t>Shipped in R-004 model evaluation suite</t>
         </is>
       </c>
     </row>

</xml_diff>